<commit_message>
feat: add end-to-end import roundtrip tests (import → sign → check)
Five new tests verify the full pipeline for each pack and profile:
- VV40 Complete (13 factors) → sign → C1+C2 pass
- NASA Complete (19 factors) → sign → C1+C2 pass
- VV40 Minimal → sign → C1+C2 pass
- NASA Minimal → sign → C1+C2 pass
- Starter xlsx → sign → C1 pass (C2 partial due to domain values)

Fixed excel_mapper to populate SHACL-required properties for evidence
sub-types (ReviewActivity.reviewer, ProcessAttestation.processType,
DeploymentRecord.deployedIn, InputPedigreeLink.sourceReference).

172 tests pass, 0 failures.
</commit_message>
<xml_diff>
--- a/tests/fixtures/import/tc06-nasa-complete-19-factors.xlsx
+++ b/tests/fixtures/import/tc06-nasa-complete-19-factors.xlsx
@@ -792,6 +792,11 @@
           <t>https://example.org/validation/tech-review</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://example.org/org/reviewer-1</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -819,6 +824,11 @@
           <t>https://example.org/validation/process-check</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://example.org/org/qa-team</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -846,6 +856,11 @@
           <t>https://example.org/validation/deploy-record</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://example.org/system/flight-test-1</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -871,6 +886,11 @@
       <c r="C7" t="inlineStr">
         <is>
           <t>https://example.org/validation/data-source</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://example.org/data/arc-jet-facility</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">

</xml_diff>